<commit_message>
changed the naming of parental/daughter to gene1/gene2
</commit_message>
<xml_diff>
--- a/data/mouseParalogStatistics.xlsx
+++ b/data/mouseParalogStatistics.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EuclidDist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EuclidDistNorm" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EuclidDistLog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PearDist" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEC" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EuclidDistNorm" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EuclidDistLog" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PearDist" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEC" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Number of Duplicates" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -474,19 +474,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1140466</v>
+        <v>251928</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>0.8158935612762657</v>
       </c>
       <c r="D2" t="n">
-        <v>61.02387853643125</v>
+        <v>0.8043952277982247</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.4904659846305596</v>
+        <v>0.06642929999908458</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>2.748648983163731e-244</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -509,19 +509,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>92258</v>
+        <v>17394</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.5838451354333868</v>
       </c>
       <c r="D3" t="n">
-        <v>50.53335292977261</v>
+        <v>0.6479097361959842</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.07152655887480211</v>
+        <v>0.1821933681268768</v>
       </c>
       <c r="F3" t="n">
-        <v>6.46391463823992e-105</v>
+        <v>1.070835514019337e-129</v>
       </c>
     </row>
   </sheetData>
@@ -592,19 +592,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>251928</v>
+        <v>1140466</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8158935612762657</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8043952277982247</v>
+        <v>1.506940359764535</v>
       </c>
       <c r="E2" t="n">
-        <v>0.06642929999908458</v>
+        <v>-0.4839282477715128</v>
       </c>
       <c r="F2" t="n">
-        <v>2.748648983163731e-244</v>
+        <v>0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -627,19 +627,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17394</v>
+        <v>92258</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5838451354333868</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6479097361959842</v>
+        <v>0.8096279674972267</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1821933681268768</v>
+        <v>-0.06961711293245124</v>
       </c>
       <c r="F3" t="n">
-        <v>1.070835514019337e-129</v>
+        <v>1.771249832769592e-99</v>
       </c>
     </row>
   </sheetData>
@@ -710,19 +710,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1140466</v>
+        <v>251928</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>0.6124181221230083</v>
       </c>
       <c r="D2" t="n">
-        <v>1.506940359764535</v>
+        <v>0.6305747835336071</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.4839282477715128</v>
+        <v>0.02179159648262379</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>7.504242238357384e-28</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -745,19 +745,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>92258</v>
+        <v>17394</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.3345333502993335</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8096279674972267</v>
+        <v>0.4851527491536364</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.06961711293245124</v>
+        <v>0.2059951748357896</v>
       </c>
       <c r="F3" t="n">
-        <v>1.771249832769592e-99</v>
+        <v>5.134032260953696e-166</v>
       </c>
     </row>
   </sheetData>
@@ -828,19 +828,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>251928</v>
+        <v>174466</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6124181221230083</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6305747835336071</v>
+        <v>0.231419861858744</v>
       </c>
       <c r="E2" t="n">
-        <v>0.02179159648262379</v>
+        <v>0.03446594086951262</v>
       </c>
       <c r="F2" t="n">
-        <v>7.504242238357384e-28</v>
+        <v>5.152118599598324e-47</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -853,7 +853,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>7.911790107124644e-31</v>
       </c>
     </row>
     <row r="3">
@@ -863,19 +863,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17394</v>
+        <v>7824</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3345333502993335</v>
+        <v>0.2142857142857143</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4851527491536364</v>
+        <v>0.19744863180446</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2059951748357896</v>
+        <v>-0.06891601366955551</v>
       </c>
       <c r="F3" t="n">
-        <v>5.134032260953696e-166</v>
+        <v>1.04660431911476e-09</v>
       </c>
     </row>
   </sheetData>
@@ -946,19 +946,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>174466</v>
+        <v>2268722</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1666666666666667</v>
+        <v>613</v>
       </c>
       <c r="D2" t="n">
-        <v>0.231419861858744</v>
+        <v>594.4276857190965</v>
       </c>
       <c r="E2" t="n">
-        <v>0.03446594086951262</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>5.152118599598324e-47</v>
+        <v>0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>7.911790107124644e-31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -981,19 +981,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7824</v>
+        <v>101852</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2142857142857143</v>
+        <v>128</v>
       </c>
       <c r="D3" t="n">
-        <v>0.19744863180446</v>
+        <v>137.8068373718729</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.06891601366955551</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>1.04660431911476e-09</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>